<commit_message>
Fix Arial on computed columns, add validation note
Post-audit fixes: explicit Arial font on every formula column (Pipeline
probability/weighted, Jobs margins, Invoices balance/status/days, Dashboard
per-line table), corrected the zero-amount status prose rule in
rs_checks.json to match the family idiom, added Arial regression checks
to post_check.py (254 passing), and wrote VALIDATION_NOTE.md.

Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_015TZgLmcfhCDvYz7RAZ9Ysf
</commit_message>
<xml_diff>
--- a/RS_Command_Center/RS_Command_Center.xlsx
+++ b/RS_Command_Center/RS_Command_Center.xlsx
@@ -195,7 +195,7 @@
     <xf numFmtId="164" fontId="5" fillId="4" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="4" fillId="5" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="11" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="4" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="4" fontId="6" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="12" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="4" fillId="5" borderId="2" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="166" fontId="14" fillId="4" borderId="0" applyProtection="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -207,10 +207,10 @@
     <xf numFmtId="4" fontId="14" fillId="4" borderId="0" applyProtection="1" pivotButton="0" quotePrefix="0" xfId="0">
       <protection locked="0" hidden="0"/>
     </xf>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="164" fontId="6" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="13" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="1" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="1" fontId="6" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="10" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="11" fillId="5" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="164" fontId="14" fillId="4" borderId="0" applyProtection="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -13847,7 +13847,7 @@
       <c r="J5" s="21" t="n">
         <v>46152</v>
       </c>
-      <c r="K5">
+      <c r="K5" s="8">
         <f>IF($F5="","",IF($I5&lt;=0,"Paid",IF(AND($J5&lt;&gt;"",TODAY()&gt;$J5),"Overdue",IF(N($G5)&gt;0,"Partial","Upcoming"))))</f>
         <v/>
       </c>
@@ -13896,7 +13896,7 @@
       <c r="J6" s="21" t="n">
         <v>46174</v>
       </c>
-      <c r="K6">
+      <c r="K6" s="8">
         <f>IF($F6="","",IF($I6&lt;=0,"Paid",IF(AND($J6&lt;&gt;"",TODAY()&gt;$J6),"Overdue",IF(N($G6)&gt;0,"Partial","Upcoming"))))</f>
         <v/>
       </c>
@@ -13945,7 +13945,7 @@
       <c r="J7" s="21" t="n">
         <v>46188</v>
       </c>
-      <c r="K7">
+      <c r="K7" s="8">
         <f>IF($F7="","",IF($I7&lt;=0,"Paid",IF(AND($J7&lt;&gt;"",TODAY()&gt;$J7),"Overdue",IF(N($G7)&gt;0,"Partial","Upcoming"))))</f>
         <v/>
       </c>
@@ -13992,7 +13992,7 @@
       <c r="J8" s="21" t="n">
         <v>46201</v>
       </c>
-      <c r="K8">
+      <c r="K8" s="8">
         <f>IF($F8="","",IF($I8&lt;=0,"Paid",IF(AND($J8&lt;&gt;"",TODAY()&gt;$J8),"Overdue",IF(N($G8)&gt;0,"Partial","Upcoming"))))</f>
         <v/>
       </c>
@@ -14041,7 +14041,7 @@
       <c r="J9" s="21" t="n">
         <v>46223</v>
       </c>
-      <c r="K9">
+      <c r="K9" s="8">
         <f>IF($F9="","",IF($I9&lt;=0,"Paid",IF(AND($J9&lt;&gt;"",TODAY()&gt;$J9),"Overdue",IF(N($G9)&gt;0,"Partial","Upcoming"))))</f>
         <v/>
       </c>
@@ -14088,7 +14088,7 @@
       <c r="J10" s="21" t="n">
         <v>46228</v>
       </c>
-      <c r="K10">
+      <c r="K10" s="8">
         <f>IF($F10="","",IF($I10&lt;=0,"Paid",IF(AND($J10&lt;&gt;"",TODAY()&gt;$J10),"Overdue",IF(N($G10)&gt;0,"Partial","Upcoming"))))</f>
         <v/>
       </c>
@@ -14115,7 +14115,7 @@
         <v/>
       </c>
       <c r="J11" s="21" t="n"/>
-      <c r="K11">
+      <c r="K11" s="8">
         <f>IF($F11="","",IF($I11&lt;=0,"Paid",IF(AND($J11&lt;&gt;"",TODAY()&gt;$J11),"Overdue",IF(N($G11)&gt;0,"Partial","Upcoming"))))</f>
         <v/>
       </c>
@@ -14138,7 +14138,7 @@
         <v/>
       </c>
       <c r="J12" s="21" t="n"/>
-      <c r="K12">
+      <c r="K12" s="8">
         <f>IF($F12="","",IF($I12&lt;=0,"Paid",IF(AND($J12&lt;&gt;"",TODAY()&gt;$J12),"Overdue",IF(N($G12)&gt;0,"Partial","Upcoming"))))</f>
         <v/>
       </c>
@@ -14161,7 +14161,7 @@
         <v/>
       </c>
       <c r="J13" s="21" t="n"/>
-      <c r="K13">
+      <c r="K13" s="8">
         <f>IF($F13="","",IF($I13&lt;=0,"Paid",IF(AND($J13&lt;&gt;"",TODAY()&gt;$J13),"Overdue",IF(N($G13)&gt;0,"Partial","Upcoming"))))</f>
         <v/>
       </c>
@@ -14184,7 +14184,7 @@
         <v/>
       </c>
       <c r="J14" s="21" t="n"/>
-      <c r="K14">
+      <c r="K14" s="8">
         <f>IF($F14="","",IF($I14&lt;=0,"Paid",IF(AND($J14&lt;&gt;"",TODAY()&gt;$J14),"Overdue",IF(N($G14)&gt;0,"Partial","Upcoming"))))</f>
         <v/>
       </c>
@@ -14207,7 +14207,7 @@
         <v/>
       </c>
       <c r="J15" s="21" t="n"/>
-      <c r="K15">
+      <c r="K15" s="8">
         <f>IF($F15="","",IF($I15&lt;=0,"Paid",IF(AND($J15&lt;&gt;"",TODAY()&gt;$J15),"Overdue",IF(N($G15)&gt;0,"Partial","Upcoming"))))</f>
         <v/>
       </c>
@@ -14230,7 +14230,7 @@
         <v/>
       </c>
       <c r="J16" s="21" t="n"/>
-      <c r="K16">
+      <c r="K16" s="8">
         <f>IF($F16="","",IF($I16&lt;=0,"Paid",IF(AND($J16&lt;&gt;"",TODAY()&gt;$J16),"Overdue",IF(N($G16)&gt;0,"Partial","Upcoming"))))</f>
         <v/>
       </c>
@@ -14253,7 +14253,7 @@
         <v/>
       </c>
       <c r="J17" s="21" t="n"/>
-      <c r="K17">
+      <c r="K17" s="8">
         <f>IF($F17="","",IF($I17&lt;=0,"Paid",IF(AND($J17&lt;&gt;"",TODAY()&gt;$J17),"Overdue",IF(N($G17)&gt;0,"Partial","Upcoming"))))</f>
         <v/>
       </c>
@@ -14276,7 +14276,7 @@
         <v/>
       </c>
       <c r="J18" s="21" t="n"/>
-      <c r="K18">
+      <c r="K18" s="8">
         <f>IF($F18="","",IF($I18&lt;=0,"Paid",IF(AND($J18&lt;&gt;"",TODAY()&gt;$J18),"Overdue",IF(N($G18)&gt;0,"Partial","Upcoming"))))</f>
         <v/>
       </c>
@@ -14299,7 +14299,7 @@
         <v/>
       </c>
       <c r="J19" s="21" t="n"/>
-      <c r="K19">
+      <c r="K19" s="8">
         <f>IF($F19="","",IF($I19&lt;=0,"Paid",IF(AND($J19&lt;&gt;"",TODAY()&gt;$J19),"Overdue",IF(N($G19)&gt;0,"Partial","Upcoming"))))</f>
         <v/>
       </c>
@@ -14322,7 +14322,7 @@
         <v/>
       </c>
       <c r="J20" s="21" t="n"/>
-      <c r="K20">
+      <c r="K20" s="8">
         <f>IF($F20="","",IF($I20&lt;=0,"Paid",IF(AND($J20&lt;&gt;"",TODAY()&gt;$J20),"Overdue",IF(N($G20)&gt;0,"Partial","Upcoming"))))</f>
         <v/>
       </c>
@@ -14345,7 +14345,7 @@
         <v/>
       </c>
       <c r="J21" s="21" t="n"/>
-      <c r="K21">
+      <c r="K21" s="8">
         <f>IF($F21="","",IF($I21&lt;=0,"Paid",IF(AND($J21&lt;&gt;"",TODAY()&gt;$J21),"Overdue",IF(N($G21)&gt;0,"Partial","Upcoming"))))</f>
         <v/>
       </c>
@@ -14368,7 +14368,7 @@
         <v/>
       </c>
       <c r="J22" s="21" t="n"/>
-      <c r="K22">
+      <c r="K22" s="8">
         <f>IF($F22="","",IF($I22&lt;=0,"Paid",IF(AND($J22&lt;&gt;"",TODAY()&gt;$J22),"Overdue",IF(N($G22)&gt;0,"Partial","Upcoming"))))</f>
         <v/>
       </c>
@@ -14391,7 +14391,7 @@
         <v/>
       </c>
       <c r="J23" s="21" t="n"/>
-      <c r="K23">
+      <c r="K23" s="8">
         <f>IF($F23="","",IF($I23&lt;=0,"Paid",IF(AND($J23&lt;&gt;"",TODAY()&gt;$J23),"Overdue",IF(N($G23)&gt;0,"Partial","Upcoming"))))</f>
         <v/>
       </c>
@@ -14414,7 +14414,7 @@
         <v/>
       </c>
       <c r="J24" s="21" t="n"/>
-      <c r="K24">
+      <c r="K24" s="8">
         <f>IF($F24="","",IF($I24&lt;=0,"Paid",IF(AND($J24&lt;&gt;"",TODAY()&gt;$J24),"Overdue",IF(N($G24)&gt;0,"Partial","Upcoming"))))</f>
         <v/>
       </c>
@@ -14437,7 +14437,7 @@
         <v/>
       </c>
       <c r="J25" s="21" t="n"/>
-      <c r="K25">
+      <c r="K25" s="8">
         <f>IF($F25="","",IF($I25&lt;=0,"Paid",IF(AND($J25&lt;&gt;"",TODAY()&gt;$J25),"Overdue",IF(N($G25)&gt;0,"Partial","Upcoming"))))</f>
         <v/>
       </c>
@@ -14460,7 +14460,7 @@
         <v/>
       </c>
       <c r="J26" s="21" t="n"/>
-      <c r="K26">
+      <c r="K26" s="8">
         <f>IF($F26="","",IF($I26&lt;=0,"Paid",IF(AND($J26&lt;&gt;"",TODAY()&gt;$J26),"Overdue",IF(N($G26)&gt;0,"Partial","Upcoming"))))</f>
         <v/>
       </c>
@@ -14483,7 +14483,7 @@
         <v/>
       </c>
       <c r="J27" s="21" t="n"/>
-      <c r="K27">
+      <c r="K27" s="8">
         <f>IF($F27="","",IF($I27&lt;=0,"Paid",IF(AND($J27&lt;&gt;"",TODAY()&gt;$J27),"Overdue",IF(N($G27)&gt;0,"Partial","Upcoming"))))</f>
         <v/>
       </c>
@@ -14506,7 +14506,7 @@
         <v/>
       </c>
       <c r="J28" s="21" t="n"/>
-      <c r="K28">
+      <c r="K28" s="8">
         <f>IF($F28="","",IF($I28&lt;=0,"Paid",IF(AND($J28&lt;&gt;"",TODAY()&gt;$J28),"Overdue",IF(N($G28)&gt;0,"Partial","Upcoming"))))</f>
         <v/>
       </c>
@@ -14529,7 +14529,7 @@
         <v/>
       </c>
       <c r="J29" s="21" t="n"/>
-      <c r="K29">
+      <c r="K29" s="8">
         <f>IF($F29="","",IF($I29&lt;=0,"Paid",IF(AND($J29&lt;&gt;"",TODAY()&gt;$J29),"Overdue",IF(N($G29)&gt;0,"Partial","Upcoming"))))</f>
         <v/>
       </c>
@@ -14552,7 +14552,7 @@
         <v/>
       </c>
       <c r="J30" s="21" t="n"/>
-      <c r="K30">
+      <c r="K30" s="8">
         <f>IF($F30="","",IF($I30&lt;=0,"Paid",IF(AND($J30&lt;&gt;"",TODAY()&gt;$J30),"Overdue",IF(N($G30)&gt;0,"Partial","Upcoming"))))</f>
         <v/>
       </c>
@@ -14575,7 +14575,7 @@
         <v/>
       </c>
       <c r="J31" s="21" t="n"/>
-      <c r="K31">
+      <c r="K31" s="8">
         <f>IF($F31="","",IF($I31&lt;=0,"Paid",IF(AND($J31&lt;&gt;"",TODAY()&gt;$J31),"Overdue",IF(N($G31)&gt;0,"Partial","Upcoming"))))</f>
         <v/>
       </c>
@@ -14598,7 +14598,7 @@
         <v/>
       </c>
       <c r="J32" s="21" t="n"/>
-      <c r="K32">
+      <c r="K32" s="8">
         <f>IF($F32="","",IF($I32&lt;=0,"Paid",IF(AND($J32&lt;&gt;"",TODAY()&gt;$J32),"Overdue",IF(N($G32)&gt;0,"Partial","Upcoming"))))</f>
         <v/>
       </c>
@@ -14621,7 +14621,7 @@
         <v/>
       </c>
       <c r="J33" s="21" t="n"/>
-      <c r="K33">
+      <c r="K33" s="8">
         <f>IF($F33="","",IF($I33&lt;=0,"Paid",IF(AND($J33&lt;&gt;"",TODAY()&gt;$J33),"Overdue",IF(N($G33)&gt;0,"Partial","Upcoming"))))</f>
         <v/>
       </c>
@@ -14644,7 +14644,7 @@
         <v/>
       </c>
       <c r="J34" s="21" t="n"/>
-      <c r="K34">
+      <c r="K34" s="8">
         <f>IF($F34="","",IF($I34&lt;=0,"Paid",IF(AND($J34&lt;&gt;"",TODAY()&gt;$J34),"Overdue",IF(N($G34)&gt;0,"Partial","Upcoming"))))</f>
         <v/>
       </c>
@@ -14667,7 +14667,7 @@
         <v/>
       </c>
       <c r="J35" s="21" t="n"/>
-      <c r="K35">
+      <c r="K35" s="8">
         <f>IF($F35="","",IF($I35&lt;=0,"Paid",IF(AND($J35&lt;&gt;"",TODAY()&gt;$J35),"Overdue",IF(N($G35)&gt;0,"Partial","Upcoming"))))</f>
         <v/>
       </c>
@@ -14690,7 +14690,7 @@
         <v/>
       </c>
       <c r="J36" s="21" t="n"/>
-      <c r="K36">
+      <c r="K36" s="8">
         <f>IF($F36="","",IF($I36&lt;=0,"Paid",IF(AND($J36&lt;&gt;"",TODAY()&gt;$J36),"Overdue",IF(N($G36)&gt;0,"Partial","Upcoming"))))</f>
         <v/>
       </c>
@@ -14713,7 +14713,7 @@
         <v/>
       </c>
       <c r="J37" s="21" t="n"/>
-      <c r="K37">
+      <c r="K37" s="8">
         <f>IF($F37="","",IF($I37&lt;=0,"Paid",IF(AND($J37&lt;&gt;"",TODAY()&gt;$J37),"Overdue",IF(N($G37)&gt;0,"Partial","Upcoming"))))</f>
         <v/>
       </c>
@@ -14736,7 +14736,7 @@
         <v/>
       </c>
       <c r="J38" s="21" t="n"/>
-      <c r="K38">
+      <c r="K38" s="8">
         <f>IF($F38="","",IF($I38&lt;=0,"Paid",IF(AND($J38&lt;&gt;"",TODAY()&gt;$J38),"Overdue",IF(N($G38)&gt;0,"Partial","Upcoming"))))</f>
         <v/>
       </c>
@@ -14759,7 +14759,7 @@
         <v/>
       </c>
       <c r="J39" s="21" t="n"/>
-      <c r="K39">
+      <c r="K39" s="8">
         <f>IF($F39="","",IF($I39&lt;=0,"Paid",IF(AND($J39&lt;&gt;"",TODAY()&gt;$J39),"Overdue",IF(N($G39)&gt;0,"Partial","Upcoming"))))</f>
         <v/>
       </c>
@@ -14782,7 +14782,7 @@
         <v/>
       </c>
       <c r="J40" s="21" t="n"/>
-      <c r="K40">
+      <c r="K40" s="8">
         <f>IF($F40="","",IF($I40&lt;=0,"Paid",IF(AND($J40&lt;&gt;"",TODAY()&gt;$J40),"Overdue",IF(N($G40)&gt;0,"Partial","Upcoming"))))</f>
         <v/>
       </c>
@@ -14805,7 +14805,7 @@
         <v/>
       </c>
       <c r="J41" s="21" t="n"/>
-      <c r="K41">
+      <c r="K41" s="8">
         <f>IF($F41="","",IF($I41&lt;=0,"Paid",IF(AND($J41&lt;&gt;"",TODAY()&gt;$J41),"Overdue",IF(N($G41)&gt;0,"Partial","Upcoming"))))</f>
         <v/>
       </c>
@@ -14828,7 +14828,7 @@
         <v/>
       </c>
       <c r="J42" s="21" t="n"/>
-      <c r="K42">
+      <c r="K42" s="8">
         <f>IF($F42="","",IF($I42&lt;=0,"Paid",IF(AND($J42&lt;&gt;"",TODAY()&gt;$J42),"Overdue",IF(N($G42)&gt;0,"Partial","Upcoming"))))</f>
         <v/>
       </c>
@@ -14851,7 +14851,7 @@
         <v/>
       </c>
       <c r="J43" s="21" t="n"/>
-      <c r="K43">
+      <c r="K43" s="8">
         <f>IF($F43="","",IF($I43&lt;=0,"Paid",IF(AND($J43&lt;&gt;"",TODAY()&gt;$J43),"Overdue",IF(N($G43)&gt;0,"Partial","Upcoming"))))</f>
         <v/>
       </c>
@@ -14874,7 +14874,7 @@
         <v/>
       </c>
       <c r="J44" s="21" t="n"/>
-      <c r="K44">
+      <c r="K44" s="8">
         <f>IF($F44="","",IF($I44&lt;=0,"Paid",IF(AND($J44&lt;&gt;"",TODAY()&gt;$J44),"Overdue",IF(N($G44)&gt;0,"Partial","Upcoming"))))</f>
         <v/>
       </c>
@@ -14897,7 +14897,7 @@
         <v/>
       </c>
       <c r="J45" s="21" t="n"/>
-      <c r="K45">
+      <c r="K45" s="8">
         <f>IF($F45="","",IF($I45&lt;=0,"Paid",IF(AND($J45&lt;&gt;"",TODAY()&gt;$J45),"Overdue",IF(N($G45)&gt;0,"Partial","Upcoming"))))</f>
         <v/>
       </c>
@@ -14920,7 +14920,7 @@
         <v/>
       </c>
       <c r="J46" s="21" t="n"/>
-      <c r="K46">
+      <c r="K46" s="8">
         <f>IF($F46="","",IF($I46&lt;=0,"Paid",IF(AND($J46&lt;&gt;"",TODAY()&gt;$J46),"Overdue",IF(N($G46)&gt;0,"Partial","Upcoming"))))</f>
         <v/>
       </c>
@@ -14943,7 +14943,7 @@
         <v/>
       </c>
       <c r="J47" s="21" t="n"/>
-      <c r="K47">
+      <c r="K47" s="8">
         <f>IF($F47="","",IF($I47&lt;=0,"Paid",IF(AND($J47&lt;&gt;"",TODAY()&gt;$J47),"Overdue",IF(N($G47)&gt;0,"Partial","Upcoming"))))</f>
         <v/>
       </c>
@@ -14966,7 +14966,7 @@
         <v/>
       </c>
       <c r="J48" s="21" t="n"/>
-      <c r="K48">
+      <c r="K48" s="8">
         <f>IF($F48="","",IF($I48&lt;=0,"Paid",IF(AND($J48&lt;&gt;"",TODAY()&gt;$J48),"Overdue",IF(N($G48)&gt;0,"Partial","Upcoming"))))</f>
         <v/>
       </c>
@@ -14989,7 +14989,7 @@
         <v/>
       </c>
       <c r="J49" s="21" t="n"/>
-      <c r="K49">
+      <c r="K49" s="8">
         <f>IF($F49="","",IF($I49&lt;=0,"Paid",IF(AND($J49&lt;&gt;"",TODAY()&gt;$J49),"Overdue",IF(N($G49)&gt;0,"Partial","Upcoming"))))</f>
         <v/>
       </c>
@@ -15012,7 +15012,7 @@
         <v/>
       </c>
       <c r="J50" s="21" t="n"/>
-      <c r="K50">
+      <c r="K50" s="8">
         <f>IF($F50="","",IF($I50&lt;=0,"Paid",IF(AND($J50&lt;&gt;"",TODAY()&gt;$J50),"Overdue",IF(N($G50)&gt;0,"Partial","Upcoming"))))</f>
         <v/>
       </c>
@@ -15035,7 +15035,7 @@
         <v/>
       </c>
       <c r="J51" s="21" t="n"/>
-      <c r="K51">
+      <c r="K51" s="8">
         <f>IF($F51="","",IF($I51&lt;=0,"Paid",IF(AND($J51&lt;&gt;"",TODAY()&gt;$J51),"Overdue",IF(N($G51)&gt;0,"Partial","Upcoming"))))</f>
         <v/>
       </c>
@@ -15058,7 +15058,7 @@
         <v/>
       </c>
       <c r="J52" s="21" t="n"/>
-      <c r="K52">
+      <c r="K52" s="8">
         <f>IF($F52="","",IF($I52&lt;=0,"Paid",IF(AND($J52&lt;&gt;"",TODAY()&gt;$J52),"Overdue",IF(N($G52)&gt;0,"Partial","Upcoming"))))</f>
         <v/>
       </c>
@@ -15081,7 +15081,7 @@
         <v/>
       </c>
       <c r="J53" s="21" t="n"/>
-      <c r="K53">
+      <c r="K53" s="8">
         <f>IF($F53="","",IF($I53&lt;=0,"Paid",IF(AND($J53&lt;&gt;"",TODAY()&gt;$J53),"Overdue",IF(N($G53)&gt;0,"Partial","Upcoming"))))</f>
         <v/>
       </c>
@@ -15104,7 +15104,7 @@
         <v/>
       </c>
       <c r="J54" s="21" t="n"/>
-      <c r="K54">
+      <c r="K54" s="8">
         <f>IF($F54="","",IF($I54&lt;=0,"Paid",IF(AND($J54&lt;&gt;"",TODAY()&gt;$J54),"Overdue",IF(N($G54)&gt;0,"Partial","Upcoming"))))</f>
         <v/>
       </c>
@@ -15127,7 +15127,7 @@
         <v/>
       </c>
       <c r="J55" s="21" t="n"/>
-      <c r="K55">
+      <c r="K55" s="8">
         <f>IF($F55="","",IF($I55&lt;=0,"Paid",IF(AND($J55&lt;&gt;"",TODAY()&gt;$J55),"Overdue",IF(N($G55)&gt;0,"Partial","Upcoming"))))</f>
         <v/>
       </c>
@@ -15150,7 +15150,7 @@
         <v/>
       </c>
       <c r="J56" s="21" t="n"/>
-      <c r="K56">
+      <c r="K56" s="8">
         <f>IF($F56="","",IF($I56&lt;=0,"Paid",IF(AND($J56&lt;&gt;"",TODAY()&gt;$J56),"Overdue",IF(N($G56)&gt;0,"Partial","Upcoming"))))</f>
         <v/>
       </c>
@@ -15173,7 +15173,7 @@
         <v/>
       </c>
       <c r="J57" s="21" t="n"/>
-      <c r="K57">
+      <c r="K57" s="8">
         <f>IF($F57="","",IF($I57&lt;=0,"Paid",IF(AND($J57&lt;&gt;"",TODAY()&gt;$J57),"Overdue",IF(N($G57)&gt;0,"Partial","Upcoming"))))</f>
         <v/>
       </c>
@@ -15196,7 +15196,7 @@
         <v/>
       </c>
       <c r="J58" s="21" t="n"/>
-      <c r="K58">
+      <c r="K58" s="8">
         <f>IF($F58="","",IF($I58&lt;=0,"Paid",IF(AND($J58&lt;&gt;"",TODAY()&gt;$J58),"Overdue",IF(N($G58)&gt;0,"Partial","Upcoming"))))</f>
         <v/>
       </c>
@@ -15219,7 +15219,7 @@
         <v/>
       </c>
       <c r="J59" s="21" t="n"/>
-      <c r="K59">
+      <c r="K59" s="8">
         <f>IF($F59="","",IF($I59&lt;=0,"Paid",IF(AND($J59&lt;&gt;"",TODAY()&gt;$J59),"Overdue",IF(N($G59)&gt;0,"Partial","Upcoming"))))</f>
         <v/>
       </c>
@@ -15242,7 +15242,7 @@
         <v/>
       </c>
       <c r="J60" s="21" t="n"/>
-      <c r="K60">
+      <c r="K60" s="8">
         <f>IF($F60="","",IF($I60&lt;=0,"Paid",IF(AND($J60&lt;&gt;"",TODAY()&gt;$J60),"Overdue",IF(N($G60)&gt;0,"Partial","Upcoming"))))</f>
         <v/>
       </c>
@@ -15265,7 +15265,7 @@
         <v/>
       </c>
       <c r="J61" s="21" t="n"/>
-      <c r="K61">
+      <c r="K61" s="8">
         <f>IF($F61="","",IF($I61&lt;=0,"Paid",IF(AND($J61&lt;&gt;"",TODAY()&gt;$J61),"Overdue",IF(N($G61)&gt;0,"Partial","Upcoming"))))</f>
         <v/>
       </c>
@@ -15288,7 +15288,7 @@
         <v/>
       </c>
       <c r="J62" s="21" t="n"/>
-      <c r="K62">
+      <c r="K62" s="8">
         <f>IF($F62="","",IF($I62&lt;=0,"Paid",IF(AND($J62&lt;&gt;"",TODAY()&gt;$J62),"Overdue",IF(N($G62)&gt;0,"Partial","Upcoming"))))</f>
         <v/>
       </c>
@@ -15311,7 +15311,7 @@
         <v/>
       </c>
       <c r="J63" s="21" t="n"/>
-      <c r="K63">
+      <c r="K63" s="8">
         <f>IF($F63="","",IF($I63&lt;=0,"Paid",IF(AND($J63&lt;&gt;"",TODAY()&gt;$J63),"Overdue",IF(N($G63)&gt;0,"Partial","Upcoming"))))</f>
         <v/>
       </c>
@@ -15334,7 +15334,7 @@
         <v/>
       </c>
       <c r="J64" s="21" t="n"/>
-      <c r="K64">
+      <c r="K64" s="8">
         <f>IF($F64="","",IF($I64&lt;=0,"Paid",IF(AND($J64&lt;&gt;"",TODAY()&gt;$J64),"Overdue",IF(N($G64)&gt;0,"Partial","Upcoming"))))</f>
         <v/>
       </c>
@@ -15357,7 +15357,7 @@
         <v/>
       </c>
       <c r="J65" s="21" t="n"/>
-      <c r="K65">
+      <c r="K65" s="8">
         <f>IF($F65="","",IF($I65&lt;=0,"Paid",IF(AND($J65&lt;&gt;"",TODAY()&gt;$J65),"Overdue",IF(N($G65)&gt;0,"Partial","Upcoming"))))</f>
         <v/>
       </c>
@@ -15380,7 +15380,7 @@
         <v/>
       </c>
       <c r="J66" s="21" t="n"/>
-      <c r="K66">
+      <c r="K66" s="8">
         <f>IF($F66="","",IF($I66&lt;=0,"Paid",IF(AND($J66&lt;&gt;"",TODAY()&gt;$J66),"Overdue",IF(N($G66)&gt;0,"Partial","Upcoming"))))</f>
         <v/>
       </c>
@@ -15403,7 +15403,7 @@
         <v/>
       </c>
       <c r="J67" s="21" t="n"/>
-      <c r="K67">
+      <c r="K67" s="8">
         <f>IF($F67="","",IF($I67&lt;=0,"Paid",IF(AND($J67&lt;&gt;"",TODAY()&gt;$J67),"Overdue",IF(N($G67)&gt;0,"Partial","Upcoming"))))</f>
         <v/>
       </c>
@@ -15426,7 +15426,7 @@
         <v/>
       </c>
       <c r="J68" s="21" t="n"/>
-      <c r="K68">
+      <c r="K68" s="8">
         <f>IF($F68="","",IF($I68&lt;=0,"Paid",IF(AND($J68&lt;&gt;"",TODAY()&gt;$J68),"Overdue",IF(N($G68)&gt;0,"Partial","Upcoming"))))</f>
         <v/>
       </c>
@@ -15449,7 +15449,7 @@
         <v/>
       </c>
       <c r="J69" s="21" t="n"/>
-      <c r="K69">
+      <c r="K69" s="8">
         <f>IF($F69="","",IF($I69&lt;=0,"Paid",IF(AND($J69&lt;&gt;"",TODAY()&gt;$J69),"Overdue",IF(N($G69)&gt;0,"Partial","Upcoming"))))</f>
         <v/>
       </c>
@@ -15472,7 +15472,7 @@
         <v/>
       </c>
       <c r="J70" s="21" t="n"/>
-      <c r="K70">
+      <c r="K70" s="8">
         <f>IF($F70="","",IF($I70&lt;=0,"Paid",IF(AND($J70&lt;&gt;"",TODAY()&gt;$J70),"Overdue",IF(N($G70)&gt;0,"Partial","Upcoming"))))</f>
         <v/>
       </c>
@@ -15495,7 +15495,7 @@
         <v/>
       </c>
       <c r="J71" s="21" t="n"/>
-      <c r="K71">
+      <c r="K71" s="8">
         <f>IF($F71="","",IF($I71&lt;=0,"Paid",IF(AND($J71&lt;&gt;"",TODAY()&gt;$J71),"Overdue",IF(N($G71)&gt;0,"Partial","Upcoming"))))</f>
         <v/>
       </c>
@@ -15518,7 +15518,7 @@
         <v/>
       </c>
       <c r="J72" s="21" t="n"/>
-      <c r="K72">
+      <c r="K72" s="8">
         <f>IF($F72="","",IF($I72&lt;=0,"Paid",IF(AND($J72&lt;&gt;"",TODAY()&gt;$J72),"Overdue",IF(N($G72)&gt;0,"Partial","Upcoming"))))</f>
         <v/>
       </c>
@@ -15541,7 +15541,7 @@
         <v/>
       </c>
       <c r="J73" s="21" t="n"/>
-      <c r="K73">
+      <c r="K73" s="8">
         <f>IF($F73="","",IF($I73&lt;=0,"Paid",IF(AND($J73&lt;&gt;"",TODAY()&gt;$J73),"Overdue",IF(N($G73)&gt;0,"Partial","Upcoming"))))</f>
         <v/>
       </c>
@@ -15564,7 +15564,7 @@
         <v/>
       </c>
       <c r="J74" s="21" t="n"/>
-      <c r="K74">
+      <c r="K74" s="8">
         <f>IF($F74="","",IF($I74&lt;=0,"Paid",IF(AND($J74&lt;&gt;"",TODAY()&gt;$J74),"Overdue",IF(N($G74)&gt;0,"Partial","Upcoming"))))</f>
         <v/>
       </c>
@@ -15587,7 +15587,7 @@
         <v/>
       </c>
       <c r="J75" s="21" t="n"/>
-      <c r="K75">
+      <c r="K75" s="8">
         <f>IF($F75="","",IF($I75&lt;=0,"Paid",IF(AND($J75&lt;&gt;"",TODAY()&gt;$J75),"Overdue",IF(N($G75)&gt;0,"Partial","Upcoming"))))</f>
         <v/>
       </c>
@@ -15610,7 +15610,7 @@
         <v/>
       </c>
       <c r="J76" s="21" t="n"/>
-      <c r="K76">
+      <c r="K76" s="8">
         <f>IF($F76="","",IF($I76&lt;=0,"Paid",IF(AND($J76&lt;&gt;"",TODAY()&gt;$J76),"Overdue",IF(N($G76)&gt;0,"Partial","Upcoming"))))</f>
         <v/>
       </c>
@@ -15633,7 +15633,7 @@
         <v/>
       </c>
       <c r="J77" s="21" t="n"/>
-      <c r="K77">
+      <c r="K77" s="8">
         <f>IF($F77="","",IF($I77&lt;=0,"Paid",IF(AND($J77&lt;&gt;"",TODAY()&gt;$J77),"Overdue",IF(N($G77)&gt;0,"Partial","Upcoming"))))</f>
         <v/>
       </c>
@@ -15656,7 +15656,7 @@
         <v/>
       </c>
       <c r="J78" s="21" t="n"/>
-      <c r="K78">
+      <c r="K78" s="8">
         <f>IF($F78="","",IF($I78&lt;=0,"Paid",IF(AND($J78&lt;&gt;"",TODAY()&gt;$J78),"Overdue",IF(N($G78)&gt;0,"Partial","Upcoming"))))</f>
         <v/>
       </c>
@@ -15679,7 +15679,7 @@
         <v/>
       </c>
       <c r="J79" s="21" t="n"/>
-      <c r="K79">
+      <c r="K79" s="8">
         <f>IF($F79="","",IF($I79&lt;=0,"Paid",IF(AND($J79&lt;&gt;"",TODAY()&gt;$J79),"Overdue",IF(N($G79)&gt;0,"Partial","Upcoming"))))</f>
         <v/>
       </c>
@@ -15702,7 +15702,7 @@
         <v/>
       </c>
       <c r="J80" s="21" t="n"/>
-      <c r="K80">
+      <c r="K80" s="8">
         <f>IF($F80="","",IF($I80&lt;=0,"Paid",IF(AND($J80&lt;&gt;"",TODAY()&gt;$J80),"Overdue",IF(N($G80)&gt;0,"Partial","Upcoming"))))</f>
         <v/>
       </c>
@@ -15725,7 +15725,7 @@
         <v/>
       </c>
       <c r="J81" s="21" t="n"/>
-      <c r="K81">
+      <c r="K81" s="8">
         <f>IF($F81="","",IF($I81&lt;=0,"Paid",IF(AND($J81&lt;&gt;"",TODAY()&gt;$J81),"Overdue",IF(N($G81)&gt;0,"Partial","Upcoming"))))</f>
         <v/>
       </c>
@@ -15748,7 +15748,7 @@
         <v/>
       </c>
       <c r="J82" s="21" t="n"/>
-      <c r="K82">
+      <c r="K82" s="8">
         <f>IF($F82="","",IF($I82&lt;=0,"Paid",IF(AND($J82&lt;&gt;"",TODAY()&gt;$J82),"Overdue",IF(N($G82)&gt;0,"Partial","Upcoming"))))</f>
         <v/>
       </c>
@@ -15771,7 +15771,7 @@
         <v/>
       </c>
       <c r="J83" s="21" t="n"/>
-      <c r="K83">
+      <c r="K83" s="8">
         <f>IF($F83="","",IF($I83&lt;=0,"Paid",IF(AND($J83&lt;&gt;"",TODAY()&gt;$J83),"Overdue",IF(N($G83)&gt;0,"Partial","Upcoming"))))</f>
         <v/>
       </c>
@@ -15794,7 +15794,7 @@
         <v/>
       </c>
       <c r="J84" s="21" t="n"/>
-      <c r="K84">
+      <c r="K84" s="8">
         <f>IF($F84="","",IF($I84&lt;=0,"Paid",IF(AND($J84&lt;&gt;"",TODAY()&gt;$J84),"Overdue",IF(N($G84)&gt;0,"Partial","Upcoming"))))</f>
         <v/>
       </c>
@@ -15817,7 +15817,7 @@
         <v/>
       </c>
       <c r="J85" s="21" t="n"/>
-      <c r="K85">
+      <c r="K85" s="8">
         <f>IF($F85="","",IF($I85&lt;=0,"Paid",IF(AND($J85&lt;&gt;"",TODAY()&gt;$J85),"Overdue",IF(N($G85)&gt;0,"Partial","Upcoming"))))</f>
         <v/>
       </c>
@@ -15840,7 +15840,7 @@
         <v/>
       </c>
       <c r="J86" s="21" t="n"/>
-      <c r="K86">
+      <c r="K86" s="8">
         <f>IF($F86="","",IF($I86&lt;=0,"Paid",IF(AND($J86&lt;&gt;"",TODAY()&gt;$J86),"Overdue",IF(N($G86)&gt;0,"Partial","Upcoming"))))</f>
         <v/>
       </c>
@@ -15863,7 +15863,7 @@
         <v/>
       </c>
       <c r="J87" s="21" t="n"/>
-      <c r="K87">
+      <c r="K87" s="8">
         <f>IF($F87="","",IF($I87&lt;=0,"Paid",IF(AND($J87&lt;&gt;"",TODAY()&gt;$J87),"Overdue",IF(N($G87)&gt;0,"Partial","Upcoming"))))</f>
         <v/>
       </c>
@@ -15886,7 +15886,7 @@
         <v/>
       </c>
       <c r="J88" s="21" t="n"/>
-      <c r="K88">
+      <c r="K88" s="8">
         <f>IF($F88="","",IF($I88&lt;=0,"Paid",IF(AND($J88&lt;&gt;"",TODAY()&gt;$J88),"Overdue",IF(N($G88)&gt;0,"Partial","Upcoming"))))</f>
         <v/>
       </c>
@@ -15909,7 +15909,7 @@
         <v/>
       </c>
       <c r="J89" s="21" t="n"/>
-      <c r="K89">
+      <c r="K89" s="8">
         <f>IF($F89="","",IF($I89&lt;=0,"Paid",IF(AND($J89&lt;&gt;"",TODAY()&gt;$J89),"Overdue",IF(N($G89)&gt;0,"Partial","Upcoming"))))</f>
         <v/>
       </c>
@@ -15932,7 +15932,7 @@
         <v/>
       </c>
       <c r="J90" s="21" t="n"/>
-      <c r="K90">
+      <c r="K90" s="8">
         <f>IF($F90="","",IF($I90&lt;=0,"Paid",IF(AND($J90&lt;&gt;"",TODAY()&gt;$J90),"Overdue",IF(N($G90)&gt;0,"Partial","Upcoming"))))</f>
         <v/>
       </c>
@@ -15955,7 +15955,7 @@
         <v/>
       </c>
       <c r="J91" s="21" t="n"/>
-      <c r="K91">
+      <c r="K91" s="8">
         <f>IF($F91="","",IF($I91&lt;=0,"Paid",IF(AND($J91&lt;&gt;"",TODAY()&gt;$J91),"Overdue",IF(N($G91)&gt;0,"Partial","Upcoming"))))</f>
         <v/>
       </c>
@@ -15978,7 +15978,7 @@
         <v/>
       </c>
       <c r="J92" s="21" t="n"/>
-      <c r="K92">
+      <c r="K92" s="8">
         <f>IF($F92="","",IF($I92&lt;=0,"Paid",IF(AND($J92&lt;&gt;"",TODAY()&gt;$J92),"Overdue",IF(N($G92)&gt;0,"Partial","Upcoming"))))</f>
         <v/>
       </c>
@@ -16001,7 +16001,7 @@
         <v/>
       </c>
       <c r="J93" s="21" t="n"/>
-      <c r="K93">
+      <c r="K93" s="8">
         <f>IF($F93="","",IF($I93&lt;=0,"Paid",IF(AND($J93&lt;&gt;"",TODAY()&gt;$J93),"Overdue",IF(N($G93)&gt;0,"Partial","Upcoming"))))</f>
         <v/>
       </c>
@@ -16024,7 +16024,7 @@
         <v/>
       </c>
       <c r="J94" s="21" t="n"/>
-      <c r="K94">
+      <c r="K94" s="8">
         <f>IF($F94="","",IF($I94&lt;=0,"Paid",IF(AND($J94&lt;&gt;"",TODAY()&gt;$J94),"Overdue",IF(N($G94)&gt;0,"Partial","Upcoming"))))</f>
         <v/>
       </c>
@@ -16047,7 +16047,7 @@
         <v/>
       </c>
       <c r="J95" s="21" t="n"/>
-      <c r="K95">
+      <c r="K95" s="8">
         <f>IF($F95="","",IF($I95&lt;=0,"Paid",IF(AND($J95&lt;&gt;"",TODAY()&gt;$J95),"Overdue",IF(N($G95)&gt;0,"Partial","Upcoming"))))</f>
         <v/>
       </c>
@@ -16070,7 +16070,7 @@
         <v/>
       </c>
       <c r="J96" s="21" t="n"/>
-      <c r="K96">
+      <c r="K96" s="8">
         <f>IF($F96="","",IF($I96&lt;=0,"Paid",IF(AND($J96&lt;&gt;"",TODAY()&gt;$J96),"Overdue",IF(N($G96)&gt;0,"Partial","Upcoming"))))</f>
         <v/>
       </c>
@@ -16093,7 +16093,7 @@
         <v/>
       </c>
       <c r="J97" s="21" t="n"/>
-      <c r="K97">
+      <c r="K97" s="8">
         <f>IF($F97="","",IF($I97&lt;=0,"Paid",IF(AND($J97&lt;&gt;"",TODAY()&gt;$J97),"Overdue",IF(N($G97)&gt;0,"Partial","Upcoming"))))</f>
         <v/>
       </c>
@@ -16116,7 +16116,7 @@
         <v/>
       </c>
       <c r="J98" s="21" t="n"/>
-      <c r="K98">
+      <c r="K98" s="8">
         <f>IF($F98="","",IF($I98&lt;=0,"Paid",IF(AND($J98&lt;&gt;"",TODAY()&gt;$J98),"Overdue",IF(N($G98)&gt;0,"Partial","Upcoming"))))</f>
         <v/>
       </c>
@@ -16139,7 +16139,7 @@
         <v/>
       </c>
       <c r="J99" s="21" t="n"/>
-      <c r="K99">
+      <c r="K99" s="8">
         <f>IF($F99="","",IF($I99&lt;=0,"Paid",IF(AND($J99&lt;&gt;"",TODAY()&gt;$J99),"Overdue",IF(N($G99)&gt;0,"Partial","Upcoming"))))</f>
         <v/>
       </c>
@@ -16162,7 +16162,7 @@
         <v/>
       </c>
       <c r="J100" s="21" t="n"/>
-      <c r="K100">
+      <c r="K100" s="8">
         <f>IF($F100="","",IF($I100&lt;=0,"Paid",IF(AND($J100&lt;&gt;"",TODAY()&gt;$J100),"Overdue",IF(N($G100)&gt;0,"Partial","Upcoming"))))</f>
         <v/>
       </c>
@@ -16185,7 +16185,7 @@
         <v/>
       </c>
       <c r="J101" s="21" t="n"/>
-      <c r="K101">
+      <c r="K101" s="8">
         <f>IF($F101="","",IF($I101&lt;=0,"Paid",IF(AND($J101&lt;&gt;"",TODAY()&gt;$J101),"Overdue",IF(N($G101)&gt;0,"Partial","Upcoming"))))</f>
         <v/>
       </c>
@@ -16208,7 +16208,7 @@
         <v/>
       </c>
       <c r="J102" s="21" t="n"/>
-      <c r="K102">
+      <c r="K102" s="8">
         <f>IF($F102="","",IF($I102&lt;=0,"Paid",IF(AND($J102&lt;&gt;"",TODAY()&gt;$J102),"Overdue",IF(N($G102)&gt;0,"Partial","Upcoming"))))</f>
         <v/>
       </c>
@@ -16231,7 +16231,7 @@
         <v/>
       </c>
       <c r="J103" s="21" t="n"/>
-      <c r="K103">
+      <c r="K103" s="8">
         <f>IF($F103="","",IF($I103&lt;=0,"Paid",IF(AND($J103&lt;&gt;"",TODAY()&gt;$J103),"Overdue",IF(N($G103)&gt;0,"Partial","Upcoming"))))</f>
         <v/>
       </c>
@@ -16254,7 +16254,7 @@
         <v/>
       </c>
       <c r="J104" s="21" t="n"/>
-      <c r="K104">
+      <c r="K104" s="8">
         <f>IF($F104="","",IF($I104&lt;=0,"Paid",IF(AND($J104&lt;&gt;"",TODAY()&gt;$J104),"Overdue",IF(N($G104)&gt;0,"Partial","Upcoming"))))</f>
         <v/>
       </c>
@@ -16277,7 +16277,7 @@
         <v/>
       </c>
       <c r="J105" s="21" t="n"/>
-      <c r="K105">
+      <c r="K105" s="8">
         <f>IF($F105="","",IF($I105&lt;=0,"Paid",IF(AND($J105&lt;&gt;"",TODAY()&gt;$J105),"Overdue",IF(N($G105)&gt;0,"Partial","Upcoming"))))</f>
         <v/>
       </c>
@@ -16300,7 +16300,7 @@
         <v/>
       </c>
       <c r="J106" s="21" t="n"/>
-      <c r="K106">
+      <c r="K106" s="8">
         <f>IF($F106="","",IF($I106&lt;=0,"Paid",IF(AND($J106&lt;&gt;"",TODAY()&gt;$J106),"Overdue",IF(N($G106)&gt;0,"Partial","Upcoming"))))</f>
         <v/>
       </c>
@@ -16323,7 +16323,7 @@
         <v/>
       </c>
       <c r="J107" s="21" t="n"/>
-      <c r="K107">
+      <c r="K107" s="8">
         <f>IF($F107="","",IF($I107&lt;=0,"Paid",IF(AND($J107&lt;&gt;"",TODAY()&gt;$J107),"Overdue",IF(N($G107)&gt;0,"Partial","Upcoming"))))</f>
         <v/>
       </c>
@@ -16346,7 +16346,7 @@
         <v/>
       </c>
       <c r="J108" s="21" t="n"/>
-      <c r="K108">
+      <c r="K108" s="8">
         <f>IF($F108="","",IF($I108&lt;=0,"Paid",IF(AND($J108&lt;&gt;"",TODAY()&gt;$J108),"Overdue",IF(N($G108)&gt;0,"Partial","Upcoming"))))</f>
         <v/>
       </c>
@@ -16369,7 +16369,7 @@
         <v/>
       </c>
       <c r="J109" s="21" t="n"/>
-      <c r="K109">
+      <c r="K109" s="8">
         <f>IF($F109="","",IF($I109&lt;=0,"Paid",IF(AND($J109&lt;&gt;"",TODAY()&gt;$J109),"Overdue",IF(N($G109)&gt;0,"Partial","Upcoming"))))</f>
         <v/>
       </c>
@@ -16392,7 +16392,7 @@
         <v/>
       </c>
       <c r="J110" s="21" t="n"/>
-      <c r="K110">
+      <c r="K110" s="8">
         <f>IF($F110="","",IF($I110&lt;=0,"Paid",IF(AND($J110&lt;&gt;"",TODAY()&gt;$J110),"Overdue",IF(N($G110)&gt;0,"Partial","Upcoming"))))</f>
         <v/>
       </c>
@@ -16415,7 +16415,7 @@
         <v/>
       </c>
       <c r="J111" s="21" t="n"/>
-      <c r="K111">
+      <c r="K111" s="8">
         <f>IF($F111="","",IF($I111&lt;=0,"Paid",IF(AND($J111&lt;&gt;"",TODAY()&gt;$J111),"Overdue",IF(N($G111)&gt;0,"Partial","Upcoming"))))</f>
         <v/>
       </c>
@@ -16438,7 +16438,7 @@
         <v/>
       </c>
       <c r="J112" s="21" t="n"/>
-      <c r="K112">
+      <c r="K112" s="8">
         <f>IF($F112="","",IF($I112&lt;=0,"Paid",IF(AND($J112&lt;&gt;"",TODAY()&gt;$J112),"Overdue",IF(N($G112)&gt;0,"Partial","Upcoming"))))</f>
         <v/>
       </c>
@@ -16461,7 +16461,7 @@
         <v/>
       </c>
       <c r="J113" s="21" t="n"/>
-      <c r="K113">
+      <c r="K113" s="8">
         <f>IF($F113="","",IF($I113&lt;=0,"Paid",IF(AND($J113&lt;&gt;"",TODAY()&gt;$J113),"Overdue",IF(N($G113)&gt;0,"Partial","Upcoming"))))</f>
         <v/>
       </c>
@@ -16484,7 +16484,7 @@
         <v/>
       </c>
       <c r="J114" s="21" t="n"/>
-      <c r="K114">
+      <c r="K114" s="8">
         <f>IF($F114="","",IF($I114&lt;=0,"Paid",IF(AND($J114&lt;&gt;"",TODAY()&gt;$J114),"Overdue",IF(N($G114)&gt;0,"Partial","Upcoming"))))</f>
         <v/>
       </c>
@@ -16507,7 +16507,7 @@
         <v/>
       </c>
       <c r="J115" s="21" t="n"/>
-      <c r="K115">
+      <c r="K115" s="8">
         <f>IF($F115="","",IF($I115&lt;=0,"Paid",IF(AND($J115&lt;&gt;"",TODAY()&gt;$J115),"Overdue",IF(N($G115)&gt;0,"Partial","Upcoming"))))</f>
         <v/>
       </c>
@@ -16530,7 +16530,7 @@
         <v/>
       </c>
       <c r="J116" s="21" t="n"/>
-      <c r="K116">
+      <c r="K116" s="8">
         <f>IF($F116="","",IF($I116&lt;=0,"Paid",IF(AND($J116&lt;&gt;"",TODAY()&gt;$J116),"Overdue",IF(N($G116)&gt;0,"Partial","Upcoming"))))</f>
         <v/>
       </c>
@@ -16553,7 +16553,7 @@
         <v/>
       </c>
       <c r="J117" s="21" t="n"/>
-      <c r="K117">
+      <c r="K117" s="8">
         <f>IF($F117="","",IF($I117&lt;=0,"Paid",IF(AND($J117&lt;&gt;"",TODAY()&gt;$J117),"Overdue",IF(N($G117)&gt;0,"Partial","Upcoming"))))</f>
         <v/>
       </c>
@@ -16576,7 +16576,7 @@
         <v/>
       </c>
       <c r="J118" s="21" t="n"/>
-      <c r="K118">
+      <c r="K118" s="8">
         <f>IF($F118="","",IF($I118&lt;=0,"Paid",IF(AND($J118&lt;&gt;"",TODAY()&gt;$J118),"Overdue",IF(N($G118)&gt;0,"Partial","Upcoming"))))</f>
         <v/>
       </c>
@@ -16599,7 +16599,7 @@
         <v/>
       </c>
       <c r="J119" s="21" t="n"/>
-      <c r="K119">
+      <c r="K119" s="8">
         <f>IF($F119="","",IF($I119&lt;=0,"Paid",IF(AND($J119&lt;&gt;"",TODAY()&gt;$J119),"Overdue",IF(N($G119)&gt;0,"Partial","Upcoming"))))</f>
         <v/>
       </c>
@@ -16622,7 +16622,7 @@
         <v/>
       </c>
       <c r="J120" s="21" t="n"/>
-      <c r="K120">
+      <c r="K120" s="8">
         <f>IF($F120="","",IF($I120&lt;=0,"Paid",IF(AND($J120&lt;&gt;"",TODAY()&gt;$J120),"Overdue",IF(N($G120)&gt;0,"Partial","Upcoming"))))</f>
         <v/>
       </c>
@@ -16645,7 +16645,7 @@
         <v/>
       </c>
       <c r="J121" s="21" t="n"/>
-      <c r="K121">
+      <c r="K121" s="8">
         <f>IF($F121="","",IF($I121&lt;=0,"Paid",IF(AND($J121&lt;&gt;"",TODAY()&gt;$J121),"Overdue",IF(N($G121)&gt;0,"Partial","Upcoming"))))</f>
         <v/>
       </c>
@@ -16668,7 +16668,7 @@
         <v/>
       </c>
       <c r="J122" s="21" t="n"/>
-      <c r="K122">
+      <c r="K122" s="8">
         <f>IF($F122="","",IF($I122&lt;=0,"Paid",IF(AND($J122&lt;&gt;"",TODAY()&gt;$J122),"Overdue",IF(N($G122)&gt;0,"Partial","Upcoming"))))</f>
         <v/>
       </c>
@@ -16691,7 +16691,7 @@
         <v/>
       </c>
       <c r="J123" s="21" t="n"/>
-      <c r="K123">
+      <c r="K123" s="8">
         <f>IF($F123="","",IF($I123&lt;=0,"Paid",IF(AND($J123&lt;&gt;"",TODAY()&gt;$J123),"Overdue",IF(N($G123)&gt;0,"Partial","Upcoming"))))</f>
         <v/>
       </c>
@@ -16714,7 +16714,7 @@
         <v/>
       </c>
       <c r="J124" s="21" t="n"/>
-      <c r="K124">
+      <c r="K124" s="8">
         <f>IF($F124="","",IF($I124&lt;=0,"Paid",IF(AND($J124&lt;&gt;"",TODAY()&gt;$J124),"Overdue",IF(N($G124)&gt;0,"Partial","Upcoming"))))</f>
         <v/>
       </c>
@@ -16737,7 +16737,7 @@
         <v/>
       </c>
       <c r="J125" s="21" t="n"/>
-      <c r="K125">
+      <c r="K125" s="8">
         <f>IF($F125="","",IF($I125&lt;=0,"Paid",IF(AND($J125&lt;&gt;"",TODAY()&gt;$J125),"Overdue",IF(N($G125)&gt;0,"Partial","Upcoming"))))</f>
         <v/>
       </c>
@@ -16760,7 +16760,7 @@
         <v/>
       </c>
       <c r="J126" s="21" t="n"/>
-      <c r="K126">
+      <c r="K126" s="8">
         <f>IF($F126="","",IF($I126&lt;=0,"Paid",IF(AND($J126&lt;&gt;"",TODAY()&gt;$J126),"Overdue",IF(N($G126)&gt;0,"Partial","Upcoming"))))</f>
         <v/>
       </c>
@@ -16783,7 +16783,7 @@
         <v/>
       </c>
       <c r="J127" s="21" t="n"/>
-      <c r="K127">
+      <c r="K127" s="8">
         <f>IF($F127="","",IF($I127&lt;=0,"Paid",IF(AND($J127&lt;&gt;"",TODAY()&gt;$J127),"Overdue",IF(N($G127)&gt;0,"Partial","Upcoming"))))</f>
         <v/>
       </c>
@@ -16806,7 +16806,7 @@
         <v/>
       </c>
       <c r="J128" s="21" t="n"/>
-      <c r="K128">
+      <c r="K128" s="8">
         <f>IF($F128="","",IF($I128&lt;=0,"Paid",IF(AND($J128&lt;&gt;"",TODAY()&gt;$J128),"Overdue",IF(N($G128)&gt;0,"Partial","Upcoming"))))</f>
         <v/>
       </c>
@@ -16829,7 +16829,7 @@
         <v/>
       </c>
       <c r="J129" s="21" t="n"/>
-      <c r="K129">
+      <c r="K129" s="8">
         <f>IF($F129="","",IF($I129&lt;=0,"Paid",IF(AND($J129&lt;&gt;"",TODAY()&gt;$J129),"Overdue",IF(N($G129)&gt;0,"Partial","Upcoming"))))</f>
         <v/>
       </c>
@@ -16852,7 +16852,7 @@
         <v/>
       </c>
       <c r="J130" s="21" t="n"/>
-      <c r="K130">
+      <c r="K130" s="8">
         <f>IF($F130="","",IF($I130&lt;=0,"Paid",IF(AND($J130&lt;&gt;"",TODAY()&gt;$J130),"Overdue",IF(N($G130)&gt;0,"Partial","Upcoming"))))</f>
         <v/>
       </c>
@@ -16875,7 +16875,7 @@
         <v/>
       </c>
       <c r="J131" s="21" t="n"/>
-      <c r="K131">
+      <c r="K131" s="8">
         <f>IF($F131="","",IF($I131&lt;=0,"Paid",IF(AND($J131&lt;&gt;"",TODAY()&gt;$J131),"Overdue",IF(N($G131)&gt;0,"Partial","Upcoming"))))</f>
         <v/>
       </c>
@@ -16898,7 +16898,7 @@
         <v/>
       </c>
       <c r="J132" s="21" t="n"/>
-      <c r="K132">
+      <c r="K132" s="8">
         <f>IF($F132="","",IF($I132&lt;=0,"Paid",IF(AND($J132&lt;&gt;"",TODAY()&gt;$J132),"Overdue",IF(N($G132)&gt;0,"Partial","Upcoming"))))</f>
         <v/>
       </c>
@@ -16921,7 +16921,7 @@
         <v/>
       </c>
       <c r="J133" s="21" t="n"/>
-      <c r="K133">
+      <c r="K133" s="8">
         <f>IF($F133="","",IF($I133&lt;=0,"Paid",IF(AND($J133&lt;&gt;"",TODAY()&gt;$J133),"Overdue",IF(N($G133)&gt;0,"Partial","Upcoming"))))</f>
         <v/>
       </c>
@@ -16944,7 +16944,7 @@
         <v/>
       </c>
       <c r="J134" s="21" t="n"/>
-      <c r="K134">
+      <c r="K134" s="8">
         <f>IF($F134="","",IF($I134&lt;=0,"Paid",IF(AND($J134&lt;&gt;"",TODAY()&gt;$J134),"Overdue",IF(N($G134)&gt;0,"Partial","Upcoming"))))</f>
         <v/>
       </c>
@@ -16967,7 +16967,7 @@
         <v/>
       </c>
       <c r="J135" s="21" t="n"/>
-      <c r="K135">
+      <c r="K135" s="8">
         <f>IF($F135="","",IF($I135&lt;=0,"Paid",IF(AND($J135&lt;&gt;"",TODAY()&gt;$J135),"Overdue",IF(N($G135)&gt;0,"Partial","Upcoming"))))</f>
         <v/>
       </c>
@@ -16990,7 +16990,7 @@
         <v/>
       </c>
       <c r="J136" s="21" t="n"/>
-      <c r="K136">
+      <c r="K136" s="8">
         <f>IF($F136="","",IF($I136&lt;=0,"Paid",IF(AND($J136&lt;&gt;"",TODAY()&gt;$J136),"Overdue",IF(N($G136)&gt;0,"Partial","Upcoming"))))</f>
         <v/>
       </c>
@@ -17013,7 +17013,7 @@
         <v/>
       </c>
       <c r="J137" s="21" t="n"/>
-      <c r="K137">
+      <c r="K137" s="8">
         <f>IF($F137="","",IF($I137&lt;=0,"Paid",IF(AND($J137&lt;&gt;"",TODAY()&gt;$J137),"Overdue",IF(N($G137)&gt;0,"Partial","Upcoming"))))</f>
         <v/>
       </c>
@@ -17036,7 +17036,7 @@
         <v/>
       </c>
       <c r="J138" s="21" t="n"/>
-      <c r="K138">
+      <c r="K138" s="8">
         <f>IF($F138="","",IF($I138&lt;=0,"Paid",IF(AND($J138&lt;&gt;"",TODAY()&gt;$J138),"Overdue",IF(N($G138)&gt;0,"Partial","Upcoming"))))</f>
         <v/>
       </c>
@@ -17059,7 +17059,7 @@
         <v/>
       </c>
       <c r="J139" s="21" t="n"/>
-      <c r="K139">
+      <c r="K139" s="8">
         <f>IF($F139="","",IF($I139&lt;=0,"Paid",IF(AND($J139&lt;&gt;"",TODAY()&gt;$J139),"Overdue",IF(N($G139)&gt;0,"Partial","Upcoming"))))</f>
         <v/>
       </c>
@@ -17082,7 +17082,7 @@
         <v/>
       </c>
       <c r="J140" s="21" t="n"/>
-      <c r="K140">
+      <c r="K140" s="8">
         <f>IF($F140="","",IF($I140&lt;=0,"Paid",IF(AND($J140&lt;&gt;"",TODAY()&gt;$J140),"Overdue",IF(N($G140)&gt;0,"Partial","Upcoming"))))</f>
         <v/>
       </c>
@@ -17105,7 +17105,7 @@
         <v/>
       </c>
       <c r="J141" s="21" t="n"/>
-      <c r="K141">
+      <c r="K141" s="8">
         <f>IF($F141="","",IF($I141&lt;=0,"Paid",IF(AND($J141&lt;&gt;"",TODAY()&gt;$J141),"Overdue",IF(N($G141)&gt;0,"Partial","Upcoming"))))</f>
         <v/>
       </c>
@@ -17128,7 +17128,7 @@
         <v/>
       </c>
       <c r="J142" s="21" t="n"/>
-      <c r="K142">
+      <c r="K142" s="8">
         <f>IF($F142="","",IF($I142&lt;=0,"Paid",IF(AND($J142&lt;&gt;"",TODAY()&gt;$J142),"Overdue",IF(N($G142)&gt;0,"Partial","Upcoming"))))</f>
         <v/>
       </c>
@@ -17151,7 +17151,7 @@
         <v/>
       </c>
       <c r="J143" s="21" t="n"/>
-      <c r="K143">
+      <c r="K143" s="8">
         <f>IF($F143="","",IF($I143&lt;=0,"Paid",IF(AND($J143&lt;&gt;"",TODAY()&gt;$J143),"Overdue",IF(N($G143)&gt;0,"Partial","Upcoming"))))</f>
         <v/>
       </c>
@@ -17174,7 +17174,7 @@
         <v/>
       </c>
       <c r="J144" s="21" t="n"/>
-      <c r="K144">
+      <c r="K144" s="8">
         <f>IF($F144="","",IF($I144&lt;=0,"Paid",IF(AND($J144&lt;&gt;"",TODAY()&gt;$J144),"Overdue",IF(N($G144)&gt;0,"Partial","Upcoming"))))</f>
         <v/>
       </c>
@@ -17197,7 +17197,7 @@
         <v/>
       </c>
       <c r="J145" s="21" t="n"/>
-      <c r="K145">
+      <c r="K145" s="8">
         <f>IF($F145="","",IF($I145&lt;=0,"Paid",IF(AND($J145&lt;&gt;"",TODAY()&gt;$J145),"Overdue",IF(N($G145)&gt;0,"Partial","Upcoming"))))</f>
         <v/>
       </c>
@@ -17220,7 +17220,7 @@
         <v/>
       </c>
       <c r="J146" s="21" t="n"/>
-      <c r="K146">
+      <c r="K146" s="8">
         <f>IF($F146="","",IF($I146&lt;=0,"Paid",IF(AND($J146&lt;&gt;"",TODAY()&gt;$J146),"Overdue",IF(N($G146)&gt;0,"Partial","Upcoming"))))</f>
         <v/>
       </c>
@@ -17243,7 +17243,7 @@
         <v/>
       </c>
       <c r="J147" s="21" t="n"/>
-      <c r="K147">
+      <c r="K147" s="8">
         <f>IF($F147="","",IF($I147&lt;=0,"Paid",IF(AND($J147&lt;&gt;"",TODAY()&gt;$J147),"Overdue",IF(N($G147)&gt;0,"Partial","Upcoming"))))</f>
         <v/>
       </c>
@@ -17266,7 +17266,7 @@
         <v/>
       </c>
       <c r="J148" s="21" t="n"/>
-      <c r="K148">
+      <c r="K148" s="8">
         <f>IF($F148="","",IF($I148&lt;=0,"Paid",IF(AND($J148&lt;&gt;"",TODAY()&gt;$J148),"Overdue",IF(N($G148)&gt;0,"Partial","Upcoming"))))</f>
         <v/>
       </c>
@@ -17289,7 +17289,7 @@
         <v/>
       </c>
       <c r="J149" s="21" t="n"/>
-      <c r="K149">
+      <c r="K149" s="8">
         <f>IF($F149="","",IF($I149&lt;=0,"Paid",IF(AND($J149&lt;&gt;"",TODAY()&gt;$J149),"Overdue",IF(N($G149)&gt;0,"Partial","Upcoming"))))</f>
         <v/>
       </c>
@@ -17312,7 +17312,7 @@
         <v/>
       </c>
       <c r="J150" s="21" t="n"/>
-      <c r="K150">
+      <c r="K150" s="8">
         <f>IF($F150="","",IF($I150&lt;=0,"Paid",IF(AND($J150&lt;&gt;"",TODAY()&gt;$J150),"Overdue",IF(N($G150)&gt;0,"Partial","Upcoming"))))</f>
         <v/>
       </c>
@@ -17335,7 +17335,7 @@
         <v/>
       </c>
       <c r="J151" s="21" t="n"/>
-      <c r="K151">
+      <c r="K151" s="8">
         <f>IF($F151="","",IF($I151&lt;=0,"Paid",IF(AND($J151&lt;&gt;"",TODAY()&gt;$J151),"Overdue",IF(N($G151)&gt;0,"Partial","Upcoming"))))</f>
         <v/>
       </c>
@@ -17358,7 +17358,7 @@
         <v/>
       </c>
       <c r="J152" s="21" t="n"/>
-      <c r="K152">
+      <c r="K152" s="8">
         <f>IF($F152="","",IF($I152&lt;=0,"Paid",IF(AND($J152&lt;&gt;"",TODAY()&gt;$J152),"Overdue",IF(N($G152)&gt;0,"Partial","Upcoming"))))</f>
         <v/>
       </c>
@@ -17381,7 +17381,7 @@
         <v/>
       </c>
       <c r="J153" s="21" t="n"/>
-      <c r="K153">
+      <c r="K153" s="8">
         <f>IF($F153="","",IF($I153&lt;=0,"Paid",IF(AND($J153&lt;&gt;"",TODAY()&gt;$J153),"Overdue",IF(N($G153)&gt;0,"Partial","Upcoming"))))</f>
         <v/>
       </c>
@@ -17404,7 +17404,7 @@
         <v/>
       </c>
       <c r="J154" s="21" t="n"/>
-      <c r="K154">
+      <c r="K154" s="8">
         <f>IF($F154="","",IF($I154&lt;=0,"Paid",IF(AND($J154&lt;&gt;"",TODAY()&gt;$J154),"Overdue",IF(N($G154)&gt;0,"Partial","Upcoming"))))</f>
         <v/>
       </c>
@@ -17427,7 +17427,7 @@
         <v/>
       </c>
       <c r="J155" s="21" t="n"/>
-      <c r="K155">
+      <c r="K155" s="8">
         <f>IF($F155="","",IF($I155&lt;=0,"Paid",IF(AND($J155&lt;&gt;"",TODAY()&gt;$J155),"Overdue",IF(N($G155)&gt;0,"Partial","Upcoming"))))</f>
         <v/>
       </c>
@@ -17450,7 +17450,7 @@
         <v/>
       </c>
       <c r="J156" s="21" t="n"/>
-      <c r="K156">
+      <c r="K156" s="8">
         <f>IF($F156="","",IF($I156&lt;=0,"Paid",IF(AND($J156&lt;&gt;"",TODAY()&gt;$J156),"Overdue",IF(N($G156)&gt;0,"Partial","Upcoming"))))</f>
         <v/>
       </c>
@@ -17473,7 +17473,7 @@
         <v/>
       </c>
       <c r="J157" s="21" t="n"/>
-      <c r="K157">
+      <c r="K157" s="8">
         <f>IF($F157="","",IF($I157&lt;=0,"Paid",IF(AND($J157&lt;&gt;"",TODAY()&gt;$J157),"Overdue",IF(N($G157)&gt;0,"Partial","Upcoming"))))</f>
         <v/>
       </c>
@@ -17496,7 +17496,7 @@
         <v/>
       </c>
       <c r="J158" s="21" t="n"/>
-      <c r="K158">
+      <c r="K158" s="8">
         <f>IF($F158="","",IF($I158&lt;=0,"Paid",IF(AND($J158&lt;&gt;"",TODAY()&gt;$J158),"Overdue",IF(N($G158)&gt;0,"Partial","Upcoming"))))</f>
         <v/>
       </c>
@@ -17519,7 +17519,7 @@
         <v/>
       </c>
       <c r="J159" s="21" t="n"/>
-      <c r="K159">
+      <c r="K159" s="8">
         <f>IF($F159="","",IF($I159&lt;=0,"Paid",IF(AND($J159&lt;&gt;"",TODAY()&gt;$J159),"Overdue",IF(N($G159)&gt;0,"Partial","Upcoming"))))</f>
         <v/>
       </c>
@@ -17542,7 +17542,7 @@
         <v/>
       </c>
       <c r="J160" s="21" t="n"/>
-      <c r="K160">
+      <c r="K160" s="8">
         <f>IF($F160="","",IF($I160&lt;=0,"Paid",IF(AND($J160&lt;&gt;"",TODAY()&gt;$J160),"Overdue",IF(N($G160)&gt;0,"Partial","Upcoming"))))</f>
         <v/>
       </c>
@@ -17565,7 +17565,7 @@
         <v/>
       </c>
       <c r="J161" s="21" t="n"/>
-      <c r="K161">
+      <c r="K161" s="8">
         <f>IF($F161="","",IF($I161&lt;=0,"Paid",IF(AND($J161&lt;&gt;"",TODAY()&gt;$J161),"Overdue",IF(N($G161)&gt;0,"Partial","Upcoming"))))</f>
         <v/>
       </c>
@@ -17588,7 +17588,7 @@
         <v/>
       </c>
       <c r="J162" s="21" t="n"/>
-      <c r="K162">
+      <c r="K162" s="8">
         <f>IF($F162="","",IF($I162&lt;=0,"Paid",IF(AND($J162&lt;&gt;"",TODAY()&gt;$J162),"Overdue",IF(N($G162)&gt;0,"Partial","Upcoming"))))</f>
         <v/>
       </c>
@@ -17611,7 +17611,7 @@
         <v/>
       </c>
       <c r="J163" s="21" t="n"/>
-      <c r="K163">
+      <c r="K163" s="8">
         <f>IF($F163="","",IF($I163&lt;=0,"Paid",IF(AND($J163&lt;&gt;"",TODAY()&gt;$J163),"Overdue",IF(N($G163)&gt;0,"Partial","Upcoming"))))</f>
         <v/>
       </c>
@@ -17634,7 +17634,7 @@
         <v/>
       </c>
       <c r="J164" s="21" t="n"/>
-      <c r="K164">
+      <c r="K164" s="8">
         <f>IF($F164="","",IF($I164&lt;=0,"Paid",IF(AND($J164&lt;&gt;"",TODAY()&gt;$J164),"Overdue",IF(N($G164)&gt;0,"Partial","Upcoming"))))</f>
         <v/>
       </c>
@@ -17657,7 +17657,7 @@
         <v/>
       </c>
       <c r="J165" s="21" t="n"/>
-      <c r="K165">
+      <c r="K165" s="8">
         <f>IF($F165="","",IF($I165&lt;=0,"Paid",IF(AND($J165&lt;&gt;"",TODAY()&gt;$J165),"Overdue",IF(N($G165)&gt;0,"Partial","Upcoming"))))</f>
         <v/>
       </c>
@@ -17680,7 +17680,7 @@
         <v/>
       </c>
       <c r="J166" s="21" t="n"/>
-      <c r="K166">
+      <c r="K166" s="8">
         <f>IF($F166="","",IF($I166&lt;=0,"Paid",IF(AND($J166&lt;&gt;"",TODAY()&gt;$J166),"Overdue",IF(N($G166)&gt;0,"Partial","Upcoming"))))</f>
         <v/>
       </c>
@@ -17703,7 +17703,7 @@
         <v/>
       </c>
       <c r="J167" s="21" t="n"/>
-      <c r="K167">
+      <c r="K167" s="8">
         <f>IF($F167="","",IF($I167&lt;=0,"Paid",IF(AND($J167&lt;&gt;"",TODAY()&gt;$J167),"Overdue",IF(N($G167)&gt;0,"Partial","Upcoming"))))</f>
         <v/>
       </c>
@@ -17726,7 +17726,7 @@
         <v/>
       </c>
       <c r="J168" s="21" t="n"/>
-      <c r="K168">
+      <c r="K168" s="8">
         <f>IF($F168="","",IF($I168&lt;=0,"Paid",IF(AND($J168&lt;&gt;"",TODAY()&gt;$J168),"Overdue",IF(N($G168)&gt;0,"Partial","Upcoming"))))</f>
         <v/>
       </c>
@@ -17749,7 +17749,7 @@
         <v/>
       </c>
       <c r="J169" s="21" t="n"/>
-      <c r="K169">
+      <c r="K169" s="8">
         <f>IF($F169="","",IF($I169&lt;=0,"Paid",IF(AND($J169&lt;&gt;"",TODAY()&gt;$J169),"Overdue",IF(N($G169)&gt;0,"Partial","Upcoming"))))</f>
         <v/>
       </c>
@@ -17772,7 +17772,7 @@
         <v/>
       </c>
       <c r="J170" s="21" t="n"/>
-      <c r="K170">
+      <c r="K170" s="8">
         <f>IF($F170="","",IF($I170&lt;=0,"Paid",IF(AND($J170&lt;&gt;"",TODAY()&gt;$J170),"Overdue",IF(N($G170)&gt;0,"Partial","Upcoming"))))</f>
         <v/>
       </c>
@@ -17795,7 +17795,7 @@
         <v/>
       </c>
       <c r="J171" s="21" t="n"/>
-      <c r="K171">
+      <c r="K171" s="8">
         <f>IF($F171="","",IF($I171&lt;=0,"Paid",IF(AND($J171&lt;&gt;"",TODAY()&gt;$J171),"Overdue",IF(N($G171)&gt;0,"Partial","Upcoming"))))</f>
         <v/>
       </c>
@@ -17818,7 +17818,7 @@
         <v/>
       </c>
       <c r="J172" s="21" t="n"/>
-      <c r="K172">
+      <c r="K172" s="8">
         <f>IF($F172="","",IF($I172&lt;=0,"Paid",IF(AND($J172&lt;&gt;"",TODAY()&gt;$J172),"Overdue",IF(N($G172)&gt;0,"Partial","Upcoming"))))</f>
         <v/>
       </c>
@@ -17841,7 +17841,7 @@
         <v/>
       </c>
       <c r="J173" s="21" t="n"/>
-      <c r="K173">
+      <c r="K173" s="8">
         <f>IF($F173="","",IF($I173&lt;=0,"Paid",IF(AND($J173&lt;&gt;"",TODAY()&gt;$J173),"Overdue",IF(N($G173)&gt;0,"Partial","Upcoming"))))</f>
         <v/>
       </c>
@@ -17864,7 +17864,7 @@
         <v/>
       </c>
       <c r="J174" s="21" t="n"/>
-      <c r="K174">
+      <c r="K174" s="8">
         <f>IF($F174="","",IF($I174&lt;=0,"Paid",IF(AND($J174&lt;&gt;"",TODAY()&gt;$J174),"Overdue",IF(N($G174)&gt;0,"Partial","Upcoming"))))</f>
         <v/>
       </c>
@@ -17887,7 +17887,7 @@
         <v/>
       </c>
       <c r="J175" s="21" t="n"/>
-      <c r="K175">
+      <c r="K175" s="8">
         <f>IF($F175="","",IF($I175&lt;=0,"Paid",IF(AND($J175&lt;&gt;"",TODAY()&gt;$J175),"Overdue",IF(N($G175)&gt;0,"Partial","Upcoming"))))</f>
         <v/>
       </c>
@@ -17910,7 +17910,7 @@
         <v/>
       </c>
       <c r="J176" s="21" t="n"/>
-      <c r="K176">
+      <c r="K176" s="8">
         <f>IF($F176="","",IF($I176&lt;=0,"Paid",IF(AND($J176&lt;&gt;"",TODAY()&gt;$J176),"Overdue",IF(N($G176)&gt;0,"Partial","Upcoming"))))</f>
         <v/>
       </c>
@@ -17933,7 +17933,7 @@
         <v/>
       </c>
       <c r="J177" s="21" t="n"/>
-      <c r="K177">
+      <c r="K177" s="8">
         <f>IF($F177="","",IF($I177&lt;=0,"Paid",IF(AND($J177&lt;&gt;"",TODAY()&gt;$J177),"Overdue",IF(N($G177)&gt;0,"Partial","Upcoming"))))</f>
         <v/>
       </c>
@@ -17956,7 +17956,7 @@
         <v/>
       </c>
       <c r="J178" s="21" t="n"/>
-      <c r="K178">
+      <c r="K178" s="8">
         <f>IF($F178="","",IF($I178&lt;=0,"Paid",IF(AND($J178&lt;&gt;"",TODAY()&gt;$J178),"Overdue",IF(N($G178)&gt;0,"Partial","Upcoming"))))</f>
         <v/>
       </c>
@@ -17979,7 +17979,7 @@
         <v/>
       </c>
       <c r="J179" s="21" t="n"/>
-      <c r="K179">
+      <c r="K179" s="8">
         <f>IF($F179="","",IF($I179&lt;=0,"Paid",IF(AND($J179&lt;&gt;"",TODAY()&gt;$J179),"Overdue",IF(N($G179)&gt;0,"Partial","Upcoming"))))</f>
         <v/>
       </c>
@@ -18002,7 +18002,7 @@
         <v/>
       </c>
       <c r="J180" s="21" t="n"/>
-      <c r="K180">
+      <c r="K180" s="8">
         <f>IF($F180="","",IF($I180&lt;=0,"Paid",IF(AND($J180&lt;&gt;"",TODAY()&gt;$J180),"Overdue",IF(N($G180)&gt;0,"Partial","Upcoming"))))</f>
         <v/>
       </c>
@@ -18025,7 +18025,7 @@
         <v/>
       </c>
       <c r="J181" s="21" t="n"/>
-      <c r="K181">
+      <c r="K181" s="8">
         <f>IF($F181="","",IF($I181&lt;=0,"Paid",IF(AND($J181&lt;&gt;"",TODAY()&gt;$J181),"Overdue",IF(N($G181)&gt;0,"Partial","Upcoming"))))</f>
         <v/>
       </c>
@@ -18048,7 +18048,7 @@
         <v/>
       </c>
       <c r="J182" s="21" t="n"/>
-      <c r="K182">
+      <c r="K182" s="8">
         <f>IF($F182="","",IF($I182&lt;=0,"Paid",IF(AND($J182&lt;&gt;"",TODAY()&gt;$J182),"Overdue",IF(N($G182)&gt;0,"Partial","Upcoming"))))</f>
         <v/>
       </c>
@@ -18071,7 +18071,7 @@
         <v/>
       </c>
       <c r="J183" s="21" t="n"/>
-      <c r="K183">
+      <c r="K183" s="8">
         <f>IF($F183="","",IF($I183&lt;=0,"Paid",IF(AND($J183&lt;&gt;"",TODAY()&gt;$J183),"Overdue",IF(N($G183)&gt;0,"Partial","Upcoming"))))</f>
         <v/>
       </c>
@@ -18094,7 +18094,7 @@
         <v/>
       </c>
       <c r="J184" s="21" t="n"/>
-      <c r="K184">
+      <c r="K184" s="8">
         <f>IF($F184="","",IF($I184&lt;=0,"Paid",IF(AND($J184&lt;&gt;"",TODAY()&gt;$J184),"Overdue",IF(N($G184)&gt;0,"Partial","Upcoming"))))</f>
         <v/>
       </c>
@@ -18117,7 +18117,7 @@
         <v/>
       </c>
       <c r="J185" s="21" t="n"/>
-      <c r="K185">
+      <c r="K185" s="8">
         <f>IF($F185="","",IF($I185&lt;=0,"Paid",IF(AND($J185&lt;&gt;"",TODAY()&gt;$J185),"Overdue",IF(N($G185)&gt;0,"Partial","Upcoming"))))</f>
         <v/>
       </c>
@@ -18140,7 +18140,7 @@
         <v/>
       </c>
       <c r="J186" s="21" t="n"/>
-      <c r="K186">
+      <c r="K186" s="8">
         <f>IF($F186="","",IF($I186&lt;=0,"Paid",IF(AND($J186&lt;&gt;"",TODAY()&gt;$J186),"Overdue",IF(N($G186)&gt;0,"Partial","Upcoming"))))</f>
         <v/>
       </c>
@@ -18163,7 +18163,7 @@
         <v/>
       </c>
       <c r="J187" s="21" t="n"/>
-      <c r="K187">
+      <c r="K187" s="8">
         <f>IF($F187="","",IF($I187&lt;=0,"Paid",IF(AND($J187&lt;&gt;"",TODAY()&gt;$J187),"Overdue",IF(N($G187)&gt;0,"Partial","Upcoming"))))</f>
         <v/>
       </c>
@@ -18186,7 +18186,7 @@
         <v/>
       </c>
       <c r="J188" s="21" t="n"/>
-      <c r="K188">
+      <c r="K188" s="8">
         <f>IF($F188="","",IF($I188&lt;=0,"Paid",IF(AND($J188&lt;&gt;"",TODAY()&gt;$J188),"Overdue",IF(N($G188)&gt;0,"Partial","Upcoming"))))</f>
         <v/>
       </c>
@@ -18209,7 +18209,7 @@
         <v/>
       </c>
       <c r="J189" s="21" t="n"/>
-      <c r="K189">
+      <c r="K189" s="8">
         <f>IF($F189="","",IF($I189&lt;=0,"Paid",IF(AND($J189&lt;&gt;"",TODAY()&gt;$J189),"Overdue",IF(N($G189)&gt;0,"Partial","Upcoming"))))</f>
         <v/>
       </c>
@@ -18232,7 +18232,7 @@
         <v/>
       </c>
       <c r="J190" s="21" t="n"/>
-      <c r="K190">
+      <c r="K190" s="8">
         <f>IF($F190="","",IF($I190&lt;=0,"Paid",IF(AND($J190&lt;&gt;"",TODAY()&gt;$J190),"Overdue",IF(N($G190)&gt;0,"Partial","Upcoming"))))</f>
         <v/>
       </c>
@@ -18255,7 +18255,7 @@
         <v/>
       </c>
       <c r="J191" s="21" t="n"/>
-      <c r="K191">
+      <c r="K191" s="8">
         <f>IF($F191="","",IF($I191&lt;=0,"Paid",IF(AND($J191&lt;&gt;"",TODAY()&gt;$J191),"Overdue",IF(N($G191)&gt;0,"Partial","Upcoming"))))</f>
         <v/>
       </c>
@@ -18278,7 +18278,7 @@
         <v/>
       </c>
       <c r="J192" s="21" t="n"/>
-      <c r="K192">
+      <c r="K192" s="8">
         <f>IF($F192="","",IF($I192&lt;=0,"Paid",IF(AND($J192&lt;&gt;"",TODAY()&gt;$J192),"Overdue",IF(N($G192)&gt;0,"Partial","Upcoming"))))</f>
         <v/>
       </c>
@@ -18301,7 +18301,7 @@
         <v/>
       </c>
       <c r="J193" s="21" t="n"/>
-      <c r="K193">
+      <c r="K193" s="8">
         <f>IF($F193="","",IF($I193&lt;=0,"Paid",IF(AND($J193&lt;&gt;"",TODAY()&gt;$J193),"Overdue",IF(N($G193)&gt;0,"Partial","Upcoming"))))</f>
         <v/>
       </c>
@@ -18324,7 +18324,7 @@
         <v/>
       </c>
       <c r="J194" s="21" t="n"/>
-      <c r="K194">
+      <c r="K194" s="8">
         <f>IF($F194="","",IF($I194&lt;=0,"Paid",IF(AND($J194&lt;&gt;"",TODAY()&gt;$J194),"Overdue",IF(N($G194)&gt;0,"Partial","Upcoming"))))</f>
         <v/>
       </c>
@@ -18347,7 +18347,7 @@
         <v/>
       </c>
       <c r="J195" s="21" t="n"/>
-      <c r="K195">
+      <c r="K195" s="8">
         <f>IF($F195="","",IF($I195&lt;=0,"Paid",IF(AND($J195&lt;&gt;"",TODAY()&gt;$J195),"Overdue",IF(N($G195)&gt;0,"Partial","Upcoming"))))</f>
         <v/>
       </c>
@@ -18370,7 +18370,7 @@
         <v/>
       </c>
       <c r="J196" s="21" t="n"/>
-      <c r="K196">
+      <c r="K196" s="8">
         <f>IF($F196="","",IF($I196&lt;=0,"Paid",IF(AND($J196&lt;&gt;"",TODAY()&gt;$J196),"Overdue",IF(N($G196)&gt;0,"Partial","Upcoming"))))</f>
         <v/>
       </c>
@@ -18393,7 +18393,7 @@
         <v/>
       </c>
       <c r="J197" s="21" t="n"/>
-      <c r="K197">
+      <c r="K197" s="8">
         <f>IF($F197="","",IF($I197&lt;=0,"Paid",IF(AND($J197&lt;&gt;"",TODAY()&gt;$J197),"Overdue",IF(N($G197)&gt;0,"Partial","Upcoming"))))</f>
         <v/>
       </c>
@@ -18416,7 +18416,7 @@
         <v/>
       </c>
       <c r="J198" s="21" t="n"/>
-      <c r="K198">
+      <c r="K198" s="8">
         <f>IF($F198="","",IF($I198&lt;=0,"Paid",IF(AND($J198&lt;&gt;"",TODAY()&gt;$J198),"Overdue",IF(N($G198)&gt;0,"Partial","Upcoming"))))</f>
         <v/>
       </c>
@@ -18439,7 +18439,7 @@
         <v/>
       </c>
       <c r="J199" s="21" t="n"/>
-      <c r="K199">
+      <c r="K199" s="8">
         <f>IF($F199="","",IF($I199&lt;=0,"Paid",IF(AND($J199&lt;&gt;"",TODAY()&gt;$J199),"Overdue",IF(N($G199)&gt;0,"Partial","Upcoming"))))</f>
         <v/>
       </c>
@@ -18462,7 +18462,7 @@
         <v/>
       </c>
       <c r="J200" s="21" t="n"/>
-      <c r="K200">
+      <c r="K200" s="8">
         <f>IF($F200="","",IF($I200&lt;=0,"Paid",IF(AND($J200&lt;&gt;"",TODAY()&gt;$J200),"Overdue",IF(N($G200)&gt;0,"Partial","Upcoming"))))</f>
         <v/>
       </c>
@@ -18485,7 +18485,7 @@
         <v/>
       </c>
       <c r="J201" s="21" t="n"/>
-      <c r="K201">
+      <c r="K201" s="8">
         <f>IF($F201="","",IF($I201&lt;=0,"Paid",IF(AND($J201&lt;&gt;"",TODAY()&gt;$J201),"Overdue",IF(N($G201)&gt;0,"Partial","Upcoming"))))</f>
         <v/>
       </c>
@@ -18508,7 +18508,7 @@
         <v/>
       </c>
       <c r="J202" s="21" t="n"/>
-      <c r="K202">
+      <c r="K202" s="8">
         <f>IF($F202="","",IF($I202&lt;=0,"Paid",IF(AND($J202&lt;&gt;"",TODAY()&gt;$J202),"Overdue",IF(N($G202)&gt;0,"Partial","Upcoming"))))</f>
         <v/>
       </c>
@@ -18531,7 +18531,7 @@
         <v/>
       </c>
       <c r="J203" s="21" t="n"/>
-      <c r="K203">
+      <c r="K203" s="8">
         <f>IF($F203="","",IF($I203&lt;=0,"Paid",IF(AND($J203&lt;&gt;"",TODAY()&gt;$J203),"Overdue",IF(N($G203)&gt;0,"Partial","Upcoming"))))</f>
         <v/>
       </c>
@@ -18554,7 +18554,7 @@
         <v/>
       </c>
       <c r="J204" s="21" t="n"/>
-      <c r="K204">
+      <c r="K204" s="8">
         <f>IF($F204="","",IF($I204&lt;=0,"Paid",IF(AND($J204&lt;&gt;"",TODAY()&gt;$J204),"Overdue",IF(N($G204)&gt;0,"Partial","Upcoming"))))</f>
         <v/>
       </c>

</xml_diff>